<commit_message>
Hoja de pedestales: d' calculado segun varilla y estribo
d' = max(rec. estribo + diametro estribo, rec. varilla) + diametro
varilla / 2, con recubrimientos minimos del ACI 318-14 Tabla
20.6.1.3.1 para concreto en contacto con el suelo (5 cm para #6 y
mayores, 4 cm para #5 y menores). Con #6 y estribo #3 da 5.95 cm,
igual que el valor que estaba capturado.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_017bbNVc9oECVNfV5wbMwybz
</commit_message>
<xml_diff>
--- a/001_H5H6_PEDESTALES_R3.2.1.xlsx
+++ b/001_H5H6_PEDESTALES_R3.2.1.xlsx
@@ -490,7 +490,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="115">
+  <cellXfs count="116">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="29" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="30" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -799,6 +799,9 @@
     </xf>
     <xf numFmtId="2" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="167" fontId="7" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -3921,8 +3924,9 @@
           <t>d' =</t>
         </is>
       </c>
-      <c r="B9" s="21" t="n">
-        <v>5.95</v>
+      <c r="B9" s="23">
+        <f>MAX(H9+INDEX(TAB_DB,MATCH(C15,LST_VAR,0)),H10)+MAX(INDEX(TAB_DB,MATCH(D13,LST_VAR,0)),IF(F13&gt;0,INDEX(TAB_DB,MATCH(G13,LST_VAR,0)),0))/2</f>
+        <v/>
       </c>
       <c r="D9" s="18" t="inlineStr">
         <is>
@@ -3933,6 +3937,15 @@
         <f>B7*B8</f>
         <v/>
       </c>
+      <c r="G9" s="13" t="inlineStr">
+        <is>
+          <t>Rec. estribo =</t>
+        </is>
+      </c>
+      <c r="H9" s="115">
+        <f>IF(INDEX(TAB_DB,MATCH(C15,LST_VAR,0))&gt;=1.9,5,4)</f>
+        <v/>
+      </c>
       <c r="Q9" s="7" t="n"/>
     </row>
     <row r="10" ht="12.75" customHeight="1">
@@ -3954,10 +3967,24 @@
         <f>E8/E9</f>
         <v/>
       </c>
+      <c r="G10" s="13" t="inlineStr">
+        <is>
+          <t>Rec. varilla =</t>
+        </is>
+      </c>
+      <c r="H10" s="115">
+        <f>IF(MAX(INDEX(TAB_DB,MATCH(D13,LST_VAR,0)),IF(F13&gt;0,INDEX(TAB_DB,MATCH(G13,LST_VAR,0)),0))&gt;=1.9,5,4)</f>
+        <v/>
+      </c>
       <c r="Q10" s="7" t="n"/>
     </row>
     <row r="11" ht="12.75" customHeight="1">
       <c r="A11" s="16" t="n"/>
+      <c r="D11" s="18" t="inlineStr">
+        <is>
+          <t>Rec. mín. ACI 318-14 T. 20.6.1.3.1 (en contacto con suelo)</t>
+        </is>
+      </c>
       <c r="Q11" s="7" t="n"/>
     </row>
     <row r="12" ht="12.75" customHeight="1">
@@ -6066,8 +6093,9 @@
           <t>d' =</t>
         </is>
       </c>
-      <c r="B9" s="21" t="n">
-        <v>5.95</v>
+      <c r="B9" s="23">
+        <f>MAX(H9+INDEX(TAB_DB,MATCH(C15,LST_VAR,0)),H10)+MAX(INDEX(TAB_DB,MATCH(D13,LST_VAR,0)),IF(F13&gt;0,INDEX(TAB_DB,MATCH(G13,LST_VAR,0)),0))/2</f>
+        <v/>
       </c>
       <c r="D9" s="18" t="inlineStr">
         <is>
@@ -6078,6 +6106,15 @@
         <f>B7*B8</f>
         <v/>
       </c>
+      <c r="G9" s="13" t="inlineStr">
+        <is>
+          <t>Rec. estribo =</t>
+        </is>
+      </c>
+      <c r="H9" s="115">
+        <f>IF(INDEX(TAB_DB,MATCH(C15,LST_VAR,0))&gt;=1.9,5,4)</f>
+        <v/>
+      </c>
       <c r="Q9" s="7" t="n"/>
     </row>
     <row r="10" ht="12.75" customHeight="1">
@@ -6099,10 +6136,24 @@
         <f>E8/E9</f>
         <v/>
       </c>
+      <c r="G10" s="13" t="inlineStr">
+        <is>
+          <t>Rec. varilla =</t>
+        </is>
+      </c>
+      <c r="H10" s="115">
+        <f>IF(MAX(INDEX(TAB_DB,MATCH(D13,LST_VAR,0)),IF(F13&gt;0,INDEX(TAB_DB,MATCH(G13,LST_VAR,0)),0))&gt;=1.9,5,4)</f>
+        <v/>
+      </c>
       <c r="Q10" s="7" t="n"/>
     </row>
     <row r="11" ht="12.75" customHeight="1">
       <c r="A11" s="16" t="n"/>
+      <c r="D11" s="18" t="inlineStr">
+        <is>
+          <t>Rec. mín. ACI 318-14 T. 20.6.1.3.1 (en contacto con suelo)</t>
+        </is>
+      </c>
       <c r="Q11" s="7" t="n"/>
     </row>
     <row r="12" ht="12.75" customHeight="1">

</xml_diff>